<commit_message>
Sources chart as red clustered columns
</commit_message>
<xml_diff>
--- a/figures/charts_tokyo.xlsx
+++ b/figures/charts_tokyo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gupta\Downloads\tokyo-uc\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{606B1B2C-177E-4F8B-9400-19CE42BF9267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D557B7B-BDFA-4E21-B4BA-65820ACD42B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{0F3B77F1-4CFD-4F87-AA5C-84E30E2038AC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{C708C515-DD71-428B-9BC8-822B47408B1D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sources" sheetId="1" r:id="rId1"/>
@@ -189,8 +189,8 @@
     <c:plotArea>
       <c:layout/>
       <c:barChart>
-        <c:barDir val="bar"/>
-        <c:grouping val="stacked"/>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
@@ -208,133 +208,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="23272E"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="2800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:srgbClr val="FFFFFF"/>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="0"/>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sources!$A$2:$A$8</c:f>
-              <c:strCache>
-                <c:ptCount val="7"/>
-                <c:pt idx="0">
-                  <c:v>Mobility</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Water</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Air &amp; climate</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Energy</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Waste</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Health</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Platform</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sources!$B$2:$B$8</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
-                <c:pt idx="0">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>1</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-08FB-44D2-87A2-475F469533D1}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sources!$C$1</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Periodic</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="8C8C8C"/>
+              <a:srgbClr val="BC002D"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -416,6 +290,135 @@
           </c:cat>
           <c:val>
             <c:numRef>
+              <c:f>Sources!$B$2:$B$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-BBA5-4DC4-AA2D-2B5320C76209}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sources!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Periodic</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="23272E"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="2800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sources!$A$2:$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>Mobility</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Water</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Air &amp; climate</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Energy</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Waste</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Health</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Platform</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
               <c:f>Sources!$C$2:$C$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
@@ -443,7 +446,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-08FB-44D2-87A2-475F469533D1}"/>
+              <c16:uniqueId val="{00000001-BBA5-4DC4-AA2D-2B5320C76209}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -563,7 +566,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-08FB-44D2-87A2-475F469533D1}"/>
+              <c16:uniqueId val="{00000002-BBA5-4DC4-AA2D-2B5320C76209}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -575,18 +578,17 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:gapWidth val="60"/>
-        <c:overlap val="100"/>
-        <c:axId val="1081338511"/>
-        <c:axId val="1081339471"/>
+        <c:gapWidth val="70"/>
+        <c:axId val="1579327647"/>
+        <c:axId val="1579332447"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1081338511"/>
+        <c:axId val="1579327647"/>
         <c:scaling>
-          <c:orientation val="maxMin"/>
+          <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="l"/>
+        <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -624,7 +626,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1081339471"/>
+        <c:crossAx val="1579332447"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -632,12 +634,12 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1081339471"/>
+        <c:axId val="1579332447"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="b"/>
+        <c:axPos val="l"/>
         <c:majorGridlines>
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
@@ -655,7 +657,7 @@
         <c:title>
           <c:tx>
             <c:rich>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
@@ -687,7 +689,7 @@
             <a:effectLst/>
           </c:spPr>
           <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr>
@@ -738,8 +740,8 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1081338511"/>
-        <c:crosses val="max"/>
+        <c:crossAx val="1579327647"/>
+        <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:spPr>
@@ -967,7 +969,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-7986-4129-9E15-9FD531BC8651}"/>
+              <c16:uniqueId val="{00000000-5325-4D32-A6CE-1BACA1FA1A62}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1081,7 +1083,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-7986-4129-9E15-9FD531BC8651}"/>
+              <c16:uniqueId val="{00000001-5325-4D32-A6CE-1BACA1FA1A62}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1201,7 +1203,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-7986-4129-9E15-9FD531BC8651}"/>
+              <c16:uniqueId val="{00000002-5325-4D32-A6CE-1BACA1FA1A62}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1327,7 +1329,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-7986-4129-9E15-9FD531BC8651}"/>
+              <c16:uniqueId val="{00000003-5325-4D32-A6CE-1BACA1FA1A62}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1447,7 +1449,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-7986-4129-9E15-9FD531BC8651}"/>
+              <c16:uniqueId val="{00000004-5325-4D32-A6CE-1BACA1FA1A62}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1461,11 +1463,11 @@
         </c:dLbls>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="1081339951"/>
-        <c:axId val="1081356751"/>
+        <c:axId val="1579334367"/>
+        <c:axId val="1579330527"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1081339951"/>
+        <c:axId val="1579334367"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1508,7 +1510,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1081356751"/>
+        <c:crossAx val="1579330527"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1516,7 +1518,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1081356751"/>
+        <c:axId val="1579330527"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1622,7 +1624,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1081339951"/>
+        <c:crossAx val="1579334367"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1777,7 +1779,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-026A-4BF8-8176-EC363974B7D6}"/>
+                <c16:uniqueId val="{00000001-F1FC-4EB2-811F-7F0381ECAC07}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1796,7 +1798,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000002-026A-4BF8-8176-EC363974B7D6}"/>
+                <c16:uniqueId val="{00000002-F1FC-4EB2-811F-7F0381ECAC07}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1815,7 +1817,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-026A-4BF8-8176-EC363974B7D6}"/>
+                <c16:uniqueId val="{00000003-F1FC-4EB2-811F-7F0381ECAC07}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1834,7 +1836,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000004-026A-4BF8-8176-EC363974B7D6}"/>
+                <c16:uniqueId val="{00000004-F1FC-4EB2-811F-7F0381ECAC07}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1853,7 +1855,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-026A-4BF8-8176-EC363974B7D6}"/>
+                <c16:uniqueId val="{00000005-F1FC-4EB2-811F-7F0381ECAC07}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1949,7 +1951,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-026A-4BF8-8176-EC363974B7D6}"/>
+              <c16:uniqueId val="{00000000-F1FC-4EB2-811F-7F0381ECAC07}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1963,11 +1965,11 @@
         </c:dLbls>
         <c:gapWidth val="50"/>
         <c:overlap val="-27"/>
-        <c:axId val="1081360111"/>
-        <c:axId val="1081360591"/>
+        <c:axId val="1579341567"/>
+        <c:axId val="1579338207"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1081360111"/>
+        <c:axId val="1579341567"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2065,7 +2067,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1081360591"/>
+        <c:crossAx val="1579338207"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2073,7 +2075,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1081360591"/>
+        <c:axId val="1579338207"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2179,7 +2181,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1081360111"/>
+        <c:crossAx val="1579341567"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2364,7 +2366,7 @@
 </file>
 
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -2568,23 +2570,22 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
         </a:schemeClr>
       </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="tx1">
             <a:lumMod val="65000"/>
             <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:downBar>
@@ -2689,8 +2690,8 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -2822,20 +2823,19 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -3896,7 +3896,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{72864324-84A5-C060-5DA2-DA4FDBA9ECB7}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{94D72E7C-4EE6-99B2-D7F8-28E988B01178}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3937,7 +3937,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BD73E744-C2CD-E5F4-54F6-6EFF396669D9}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{250AEA6B-187D-8351-4415-3E14C2A35336}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3978,7 +3978,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AF3A08A9-5A4F-24FA-D17D-BAF26B7C97C5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{129F70A2-C8F1-3976-67BB-D1E5503462E0}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4315,7 +4315,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A10CDC99-A52A-4B17-A744-9D62AA2385D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F02C47C-10CD-4EC8-BE95-E67FBBB8F690}">
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -4420,7 +4420,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43AC718B-F51F-4BF7-965A-C2C2FE7C342C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E82ECCF-2B8F-4DE1-A747-59107CD173E0}">
   <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -4534,7 +4534,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1D3D776-FC01-4AD8-9694-E38B8627A518}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{863C21CB-7BAC-4634-9EBF-0B9D3F028580}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>

</xml_diff>

<commit_message>
SmaGO loop diagram; initiatives chart updated with Hachi-san-Po; README lists all three diagrams
</commit_message>
<xml_diff>
--- a/figures/charts_tokyo.xlsx
+++ b/figures/charts_tokyo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gupta\Downloads\tokyo-uc\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D557B7B-BDFA-4E21-B4BA-65820ACD42B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ECD52590-5A4C-4FFB-A7D5-1E5EA60F6AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{C708C515-DD71-428B-9BC8-822B47408B1D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{35E4FC8D-F197-4791-AA1D-5777FE07D8D4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sources" sheetId="1" r:id="rId1"/>
@@ -317,7 +317,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-BBA5-4DC4-AA2D-2B5320C76209}"/>
+              <c16:uniqueId val="{00000000-3DEE-45AC-8690-37653418E1F5}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -446,7 +446,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-BBA5-4DC4-AA2D-2B5320C76209}"/>
+              <c16:uniqueId val="{00000001-3DEE-45AC-8690-37653418E1F5}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -566,7 +566,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-BBA5-4DC4-AA2D-2B5320C76209}"/>
+              <c16:uniqueId val="{00000002-3DEE-45AC-8690-37653418E1F5}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -579,11 +579,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="70"/>
-        <c:axId val="1579327647"/>
-        <c:axId val="1579332447"/>
+        <c:axId val="1062306560"/>
+        <c:axId val="1062250880"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1579327647"/>
+        <c:axId val="1062306560"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -626,7 +626,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1579332447"/>
+        <c:crossAx val="1062250880"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -634,7 +634,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1579332447"/>
+        <c:axId val="1062250880"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -740,7 +740,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1579327647"/>
+        <c:crossAx val="1062306560"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -969,7 +969,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-5325-4D32-A6CE-1BACA1FA1A62}"/>
+              <c16:uniqueId val="{00000000-00CD-4128-92ED-CC3F6D22987A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1083,7 +1083,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-5325-4D32-A6CE-1BACA1FA1A62}"/>
+              <c16:uniqueId val="{00000001-00CD-4128-92ED-CC3F6D22987A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1198,12 +1198,15 @@
                 <c:pt idx="4">
                   <c:v>2</c:v>
                 </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-5325-4D32-A6CE-1BACA1FA1A62}"/>
+              <c16:uniqueId val="{00000002-00CD-4128-92ED-CC3F6D22987A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1329,7 +1332,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-5325-4D32-A6CE-1BACA1FA1A62}"/>
+              <c16:uniqueId val="{00000003-00CD-4128-92ED-CC3F6D22987A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1449,7 +1452,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-5325-4D32-A6CE-1BACA1FA1A62}"/>
+              <c16:uniqueId val="{00000004-00CD-4128-92ED-CC3F6D22987A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1463,11 +1466,11 @@
         </c:dLbls>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="1579334367"/>
-        <c:axId val="1579330527"/>
+        <c:axId val="1062253280"/>
+        <c:axId val="1062251840"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1579334367"/>
+        <c:axId val="1062253280"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1510,7 +1513,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1579330527"/>
+        <c:crossAx val="1062251840"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1518,7 +1521,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1579330527"/>
+        <c:axId val="1062251840"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1624,7 +1627,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1579334367"/>
+        <c:crossAx val="1062253280"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1779,7 +1782,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-F1FC-4EB2-811F-7F0381ECAC07}"/>
+                <c16:uniqueId val="{00000001-C44A-4335-9850-5C83A468FAEC}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1798,7 +1801,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000002-F1FC-4EB2-811F-7F0381ECAC07}"/>
+                <c16:uniqueId val="{00000002-C44A-4335-9850-5C83A468FAEC}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1817,7 +1820,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-F1FC-4EB2-811F-7F0381ECAC07}"/>
+                <c16:uniqueId val="{00000003-C44A-4335-9850-5C83A468FAEC}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1836,7 +1839,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000004-F1FC-4EB2-811F-7F0381ECAC07}"/>
+                <c16:uniqueId val="{00000004-C44A-4335-9850-5C83A468FAEC}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1855,7 +1858,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-F1FC-4EB2-811F-7F0381ECAC07}"/>
+                <c16:uniqueId val="{00000005-C44A-4335-9850-5C83A468FAEC}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1951,7 +1954,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-F1FC-4EB2-811F-7F0381ECAC07}"/>
+              <c16:uniqueId val="{00000000-C44A-4335-9850-5C83A468FAEC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1965,11 +1968,11 @@
         </c:dLbls>
         <c:gapWidth val="50"/>
         <c:overlap val="-27"/>
-        <c:axId val="1579341567"/>
-        <c:axId val="1579338207"/>
+        <c:axId val="1062245120"/>
+        <c:axId val="1062260000"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1579341567"/>
+        <c:axId val="1062245120"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2067,7 +2070,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1579338207"/>
+        <c:crossAx val="1062260000"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2075,7 +2078,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1579338207"/>
+        <c:axId val="1062260000"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2181,7 +2184,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1579341567"/>
+        <c:crossAx val="1062245120"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3896,7 +3899,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{94D72E7C-4EE6-99B2-D7F8-28E988B01178}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C155AD0-8B80-168B-3182-D64D4FCB83C1}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3937,7 +3940,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{250AEA6B-187D-8351-4415-3E14C2A35336}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{215C4963-C2EE-C611-AF53-FF9790C6520D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3978,7 +3981,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{129F70A2-C8F1-3976-67BB-D1E5503462E0}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0576C94E-A117-80F1-985E-C26FC35C1017}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4315,7 +4318,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F02C47C-10CD-4EC8-BE95-E67FBBB8F690}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA5B9F0C-70AA-467F-9382-9487D45EDE7B}">
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -4420,7 +4423,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E82ECCF-2B8F-4DE1-A747-59107CD173E0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{905B37DC-31E3-4B76-9894-A20766DBC184}">
   <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -4511,6 +4514,9 @@
       </c>
       <c r="C7">
         <v>2</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
       </c>
       <c r="E7">
         <v>5</v>
@@ -4534,7 +4540,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{863C21CB-7BAC-4634-9EBF-0B9D3F028580}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8510E441-55D9-4E2F-8E28-E044BC474C3B}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Initiatives chart: Hachi-san-Po counted as Enabler, as in the report table
</commit_message>
<xml_diff>
--- a/figures/charts_tokyo.xlsx
+++ b/figures/charts_tokyo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gupta\Downloads\tokyo-uc\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ECD52590-5A4C-4FFB-A7D5-1E5EA60F6AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ED74F399-FA4E-419D-8D0F-7BDCC8AA91A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{35E4FC8D-F197-4791-AA1D-5777FE07D8D4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{DB9E2796-BF62-4B2C-BA6D-6011A3A5DDF8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sources" sheetId="1" r:id="rId1"/>
@@ -317,7 +317,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-3DEE-45AC-8690-37653418E1F5}"/>
+              <c16:uniqueId val="{00000000-61AA-403C-9A30-CE2A413DB59E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -446,7 +446,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-3DEE-45AC-8690-37653418E1F5}"/>
+              <c16:uniqueId val="{00000001-61AA-403C-9A30-CE2A413DB59E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -566,7 +566,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-3DEE-45AC-8690-37653418E1F5}"/>
+              <c16:uniqueId val="{00000002-61AA-403C-9A30-CE2A413DB59E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -579,11 +579,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="70"/>
-        <c:axId val="1062306560"/>
-        <c:axId val="1062250880"/>
+        <c:axId val="1699721391"/>
+        <c:axId val="1699725231"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1062306560"/>
+        <c:axId val="1699721391"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -626,7 +626,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1062250880"/>
+        <c:crossAx val="1699725231"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -634,7 +634,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1062250880"/>
+        <c:axId val="1699725231"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -740,7 +740,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1062306560"/>
+        <c:crossAx val="1699721391"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -969,7 +969,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-00CD-4128-92ED-CC3F6D22987A}"/>
+              <c16:uniqueId val="{00000000-D41D-48A0-8991-515FCEACECFD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1083,7 +1083,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-00CD-4128-92ED-CC3F6D22987A}"/>
+              <c16:uniqueId val="{00000001-D41D-48A0-8991-515FCEACECFD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1198,15 +1198,12 @@
                 <c:pt idx="4">
                   <c:v>2</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>1</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-00CD-4128-92ED-CC3F6D22987A}"/>
+              <c16:uniqueId val="{00000002-D41D-48A0-8991-515FCEACECFD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1332,7 +1329,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-00CD-4128-92ED-CC3F6D22987A}"/>
+              <c16:uniqueId val="{00000003-D41D-48A0-8991-515FCEACECFD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1444,6 +1441,9 @@
                 <c:pt idx="4">
                   <c:v>1</c:v>
                 </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
                 <c:pt idx="6">
                   <c:v>4</c:v>
                 </c:pt>
@@ -1452,7 +1452,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-00CD-4128-92ED-CC3F6D22987A}"/>
+              <c16:uniqueId val="{00000004-D41D-48A0-8991-515FCEACECFD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1466,11 +1466,11 @@
         </c:dLbls>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="1062253280"/>
-        <c:axId val="1062251840"/>
+        <c:axId val="1699733391"/>
+        <c:axId val="1699690671"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1062253280"/>
+        <c:axId val="1699733391"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1513,7 +1513,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1062251840"/>
+        <c:crossAx val="1699690671"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1521,7 +1521,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1062251840"/>
+        <c:axId val="1699690671"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1627,7 +1627,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1062253280"/>
+        <c:crossAx val="1699733391"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1782,7 +1782,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-C44A-4335-9850-5C83A468FAEC}"/>
+                <c16:uniqueId val="{00000001-5356-4EF0-8EA0-670CE8E06928}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1801,7 +1801,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000002-C44A-4335-9850-5C83A468FAEC}"/>
+                <c16:uniqueId val="{00000002-5356-4EF0-8EA0-670CE8E06928}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1820,7 +1820,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-C44A-4335-9850-5C83A468FAEC}"/>
+                <c16:uniqueId val="{00000003-5356-4EF0-8EA0-670CE8E06928}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1839,7 +1839,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000004-C44A-4335-9850-5C83A468FAEC}"/>
+                <c16:uniqueId val="{00000004-5356-4EF0-8EA0-670CE8E06928}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1858,7 +1858,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-C44A-4335-9850-5C83A468FAEC}"/>
+                <c16:uniqueId val="{00000005-5356-4EF0-8EA0-670CE8E06928}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1954,7 +1954,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C44A-4335-9850-5C83A468FAEC}"/>
+              <c16:uniqueId val="{00000000-5356-4EF0-8EA0-670CE8E06928}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1968,11 +1968,11 @@
         </c:dLbls>
         <c:gapWidth val="50"/>
         <c:overlap val="-27"/>
-        <c:axId val="1062245120"/>
-        <c:axId val="1062260000"/>
+        <c:axId val="784966016"/>
+        <c:axId val="784972256"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1062245120"/>
+        <c:axId val="784966016"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2070,7 +2070,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1062260000"/>
+        <c:crossAx val="784972256"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2078,7 +2078,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1062260000"/>
+        <c:axId val="784972256"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2184,7 +2184,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1062245120"/>
+        <c:crossAx val="784966016"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3899,7 +3899,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C155AD0-8B80-168B-3182-D64D4FCB83C1}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{573D2CFD-3FD6-B034-4240-67799342F7FC}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3940,7 +3940,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{215C4963-C2EE-C611-AF53-FF9790C6520D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4DE2C525-964D-A70A-CC22-B7435738BC0E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3981,7 +3981,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0576C94E-A117-80F1-985E-C26FC35C1017}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4929903C-AA93-0556-8B9A-8D746CB06749}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4318,7 +4318,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA5B9F0C-70AA-467F-9382-9487D45EDE7B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39FA07EB-719E-426E-9D6C-5ADA49861636}">
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -4423,7 +4423,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{905B37DC-31E3-4B76-9894-A20766DBC184}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8A264B9-AC2A-440E-83E5-B06591B73F02}">
   <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -4515,11 +4515,11 @@
       <c r="C7">
         <v>2</v>
       </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
       <c r="E7">
         <v>5</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -4540,7 +4540,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8510E441-55D9-4E2F-8E28-E044BC474C3B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DB4A966-3DDA-456C-94C8-0E74B606E73C}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>

</xml_diff>